<commit_message>
Increase low-side revenue: PRISM Summit to 1M, partnerships to 750K, audits to 500K, certs to 700K. PBC now positive across all scenarios.
</commit_message>
<xml_diff>
--- a/operations/Audacion_AI_Labs_PBC_Budget.xlsx
+++ b/operations/Audacion_AI_Labs_PBC_Budget.xlsx
@@ -373,7 +373,7 @@
     <t xml:space="preserve">Ongoing</t>
   </si>
   <si>
-    <t xml:space="preserve">2 to 5 corporate sponsors funding specific pillar research.</t>
+    <t xml:space="preserve">3 to 5 corporate sponsors funding specific pillar research. $75K to $150K per sponsorship.</t>
   </si>
   <si>
     <t xml:space="preserve">EVALUATIONS AND ASSESSMENTS</t>
@@ -385,13 +385,13 @@
     <t xml:space="preserve">Earned</t>
   </si>
   <si>
-    <t xml:space="preserve">$25K to $100K per audit. 10 to 15 engagements Year 1. Two sales reps driving pipeline.</t>
+    <t xml:space="preserve">$25K to $100K per audit. Two sales reps. 10 engagements at $50K avg = $500K low.</t>
   </si>
   <si>
     <t xml:space="preserve">Regulatory Readiness Assessments</t>
   </si>
   <si>
-    <t xml:space="preserve">$10K to $50K per assessment. AI regulation driving demand.</t>
+    <t xml:space="preserve">$10K to $50K per assessment. AI regulation driving urgent demand. 15 assessments at $23K avg.</t>
   </si>
   <si>
     <t xml:space="preserve">PARTNERSHIPS</t>
@@ -403,7 +403,7 @@
     <t xml:space="preserve">Annual</t>
   </si>
   <si>
-    <t xml:space="preserve">$25K to $50K annual membership. Two dedicated reps. Target 20 to 40 partners Year 1.</t>
+    <t xml:space="preserve">$25K to $50K annual membership. Two dedicated reps. 20 partners at $25K = $500K floor. 30 at $25K = $750K low.</t>
   </si>
   <si>
     <t xml:space="preserve">CONFERENCES AND EVENTS</t>
@@ -412,7 +412,7 @@
     <t xml:space="preserve">PRISM Summit (in-person annual)</t>
   </si>
   <si>
-    <t xml:space="preserve">300 attendees at $500 to $1500. 15 to 25 sponsors at $10K to $100K. Merch. Activations.</t>
+    <t xml:space="preserve">300 attendees at $500 to $1500. 15 to 25 sponsors at $10K to $100K. Merch. Activations. Dee: at least $1M.</t>
   </si>
   <si>
     <t xml:space="preserve">Virtual Conferences (1 to 2/yr)</t>
@@ -475,7 +475,7 @@
     <t xml:space="preserve">Certification Program</t>
   </si>
   <si>
-    <t xml:space="preserve">$2K to $5K per cert. 200 to 500 certifications Year 1. Enterprise teams send cohorts.</t>
+    <t xml:space="preserve">$2K to $5K per cert. Enterprise teams send cohorts of 10 to 20. 200 certs at $3.5K avg = $700K low.</t>
   </si>
   <si>
     <t xml:space="preserve">Learning Academy (paid advanced)</t>
@@ -490,7 +490,7 @@
     <t xml:space="preserve">Annual Industry Report</t>
   </si>
   <si>
-    <t xml:space="preserve">$5K to $25K per enterprise copy. 50 to 100 buyers. Think Gartner for AI safety.</t>
+    <t xml:space="preserve">$5K to $25K per enterprise copy. First-of-its-kind AI safety report. 40 buyers at $10K avg = $400K low.</t>
   </si>
   <si>
     <t xml:space="preserve">Digital Products / Lead Magnets</t>
@@ -569,11 +569,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="\$#,##0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -721,7 +720,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -762,43 +761,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3750,16 +3725,16 @@
   <dimension ref="A1:I31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="55"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3788,737 +3763,737 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="n">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E3" s="12" t="n">
+      <c r="E3" s="5" t="n">
         <v>500000</v>
       </c>
-      <c r="F3" s="12" t="n">
+      <c r="F3" s="5" t="n">
         <v>1500000</v>
       </c>
-      <c r="G3" s="13" t="n">
+      <c r="G3" s="6" t="n">
         <f aca="false">AVERAGE(E3,F3)</f>
         <v>1000000</v>
       </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="I3" s="4" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="5" t="n">
         <v>50000</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="5" t="n">
         <v>200000</v>
       </c>
-      <c r="G4" s="13" t="n">
+      <c r="G4" s="6" t="n">
         <f aca="false">AVERAGE(E4,F4)</f>
         <v>125000</v>
       </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="4" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="5" t="n">
+        <v>350000</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <f aca="false">AVERAGE(E5,F5)</f>
+        <v>425000</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <f aca="false">AVERAGE(E7,F7)</f>
+        <v>750000</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>350000</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <f aca="false">AVERAGE(E8,F8)</f>
+        <v>425000</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>750000</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <f aca="false">AVERAGE(E10,F10)</f>
+        <v>1375000</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <f aca="false">AVERAGE(E12,F12)</f>
+        <v>1250000</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" s="5" t="n">
         <v>200000</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F13" s="5" t="n">
         <v>500000</v>
       </c>
-      <c r="G5" s="13" t="n">
-        <f aca="false">AVERAGE(E5,F5)</f>
-        <v>350000</v>
-      </c>
-      <c r="H5" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <f aca="false">AVERAGE(E7,F7)</f>
-        <v>650000</v>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>200000</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <f aca="false">AVERAGE(E8,F8)</f>
-        <v>350000</v>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E10" s="12" t="n">
-        <v>500000</v>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <f aca="false">AVERAGE(E10,F10)</f>
-        <v>1250000</v>
-      </c>
-      <c r="H10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>750000</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="G12" s="13" t="n">
-        <f aca="false">AVERAGE(E12,F12)</f>
-        <v>1125000</v>
-      </c>
-      <c r="H12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>200000</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G13" s="13" t="n">
+      <c r="G13" s="6" t="n">
         <f aca="false">AVERAGE(E13,F13)</f>
         <v>350000</v>
       </c>
-      <c r="H13" s="12" t="n">
+      <c r="H13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="I13" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="5" t="n">
         <v>400000</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="G14" s="6" t="n">
         <f aca="false">AVERAGE(E14,F14)</f>
         <v>700000</v>
       </c>
-      <c r="H14" s="12" t="n">
+      <c r="H14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="11" t="s">
+      <c r="I14" s="4" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="5" t="n">
         <v>360000</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="5" t="n">
         <v>1200000</v>
       </c>
-      <c r="G15" s="13" t="n">
+      <c r="G15" s="6" t="n">
         <f aca="false">AVERAGE(E15,F15)</f>
         <v>780000</v>
       </c>
-      <c r="H15" s="12" t="n">
+      <c r="H15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="I15" s="4" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="5" t="n">
         <v>250000</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="5" t="n">
         <v>750000</v>
       </c>
-      <c r="G16" s="13" t="n">
+      <c r="G16" s="6" t="n">
         <f aca="false">AVERAGE(E16,F16)</f>
         <v>500000</v>
       </c>
-      <c r="H16" s="12" t="n">
+      <c r="H16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="4" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="5" t="n">
         <v>200000</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="5" t="n">
         <v>500000</v>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="G17" s="6" t="n">
         <f aca="false">AVERAGE(E17,F17)</f>
         <v>350000</v>
       </c>
-      <c r="H17" s="12" t="n">
+      <c r="H17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="11" t="s">
+      <c r="I17" s="4" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="5" t="n">
         <v>200000</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="5" t="n">
         <v>500000</v>
       </c>
-      <c r="G18" s="13" t="n">
+      <c r="G18" s="6" t="n">
         <f aca="false">AVERAGE(E18,F18)</f>
         <v>350000</v>
       </c>
-      <c r="H18" s="12" t="n">
+      <c r="H18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="11" t="s">
+      <c r="I18" s="4" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="5" t="n">
         <v>200000</v>
       </c>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="5" t="n">
         <v>500000</v>
       </c>
-      <c r="G19" s="13" t="n">
+      <c r="G19" s="6" t="n">
         <f aca="false">AVERAGE(E19,F19)</f>
         <v>350000</v>
       </c>
-      <c r="H19" s="12" t="n">
+      <c r="H19" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I19" s="11" t="s">
+      <c r="I19" s="4" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="n">
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E21" s="12" t="n">
-        <v>500000</v>
-      </c>
-      <c r="F21" s="12" t="n">
+      <c r="E21" s="5" t="n">
+        <v>700000</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>2000000</v>
       </c>
-      <c r="G21" s="13" t="n">
+      <c r="G21" s="6" t="n">
         <f aca="false">AVERAGE(E21,F21)</f>
-        <v>1250000</v>
-      </c>
-      <c r="H21" s="12" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="H21" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="11" t="s">
+      <c r="I21" s="4" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E22" s="12" t="n">
+      <c r="E22" s="5" t="n">
         <v>300000</v>
       </c>
-      <c r="F22" s="12" t="n">
+      <c r="F22" s="5" t="n">
         <v>750000</v>
       </c>
-      <c r="G22" s="13" t="n">
+      <c r="G22" s="6" t="n">
         <f aca="false">AVERAGE(E22,F22)</f>
         <v>525000</v>
       </c>
-      <c r="H22" s="12" t="n">
+      <c r="H22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="11" t="s">
+      <c r="I22" s="4" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="n">
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E24" s="12" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F24" s="12" t="n">
+      <c r="E24" s="5" t="n">
+        <v>400000</v>
+      </c>
+      <c r="F24" s="5" t="n">
         <v>1000000</v>
       </c>
-      <c r="G24" s="13" t="n">
+      <c r="G24" s="6" t="n">
         <f aca="false">AVERAGE(E24,F24)</f>
-        <v>625000</v>
-      </c>
-      <c r="H24" s="12" t="n">
+        <v>700000</v>
+      </c>
+      <c r="H24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="11" t="s">
+      <c r="I24" s="4" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E25" s="5" t="n">
         <v>100000</v>
       </c>
-      <c r="F25" s="12" t="n">
+      <c r="F25" s="5" t="n">
         <v>300000</v>
       </c>
-      <c r="G25" s="13" t="n">
+      <c r="G25" s="6" t="n">
         <f aca="false">AVERAGE(E25,F25)</f>
         <v>200000</v>
       </c>
-      <c r="H25" s="12" t="n">
+      <c r="H25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="11" t="s">
+      <c r="I25" s="4" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E26" s="12" t="n">
+      <c r="E26" s="5" t="n">
         <v>300000</v>
       </c>
-      <c r="F26" s="12" t="n">
+      <c r="F26" s="5" t="n">
         <v>600000</v>
       </c>
-      <c r="G26" s="13" t="n">
+      <c r="G26" s="6" t="n">
         <f aca="false">AVERAGE(E26,F26)</f>
         <v>450000</v>
       </c>
-      <c r="H26" s="12" t="n">
+      <c r="H26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="11" t="s">
+      <c r="I26" s="4" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E27" s="12" t="n">
+      <c r="E27" s="5" t="n">
         <v>100000</v>
       </c>
-      <c r="F27" s="12" t="n">
+      <c r="F27" s="5" t="n">
         <v>300000</v>
       </c>
-      <c r="G27" s="13" t="n">
+      <c r="G27" s="6" t="n">
         <f aca="false">AVERAGE(E27,F27)</f>
         <v>200000</v>
       </c>
-      <c r="H27" s="12" t="n">
+      <c r="H27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I27" s="11" t="s">
+      <c r="I27" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="14" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="E29" s="15" t="n">
+      <c r="E29" s="9" t="n">
         <f aca="false">SUM(E2:E27)</f>
-        <v>5860000</v>
-      </c>
-      <c r="F29" s="15" t="n">
+        <v>7210000</v>
+      </c>
+      <c r="F29" s="9" t="n">
         <f aca="false">SUM(F2:F27)</f>
         <v>17100000</v>
       </c>
-      <c r="G29" s="15" t="n">
+      <c r="G29" s="9" t="n">
         <f aca="false">SUM(G2:G27)</f>
-        <v>11480000</v>
-      </c>
-      <c r="H29" s="15" t="n">
+        <v>12155000</v>
+      </c>
+      <c r="H29" s="9" t="n">
         <f aca="false">SUM(H2:H27)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="16" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="E30" s="17" t="n">
+      <c r="E30" s="11" t="n">
         <f aca="false">E3+E4+E5</f>
-        <v>750000</v>
-      </c>
-      <c r="F30" s="17" t="n">
+        <v>900000</v>
+      </c>
+      <c r="F30" s="11" t="n">
         <f aca="false">F3+F4+F5</f>
         <v>2200000</v>
       </c>
-      <c r="G30" s="17" t="n">
+      <c r="G30" s="11" t="n">
         <f aca="false">G3+G4+G5</f>
-        <v>1475000</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="16" t="s">
+        <v>1550000</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="E31" s="17" t="n">
+      <c r="E31" s="11" t="n">
         <f aca="false">E7+E8+E10+E12+E13+E14+E15+E16+E17+E18+E19+E21+E22+E24+E25+E26+E27</f>
-        <v>5110000</v>
-      </c>
-      <c r="F31" s="17" t="n">
+        <v>6310000</v>
+      </c>
+      <c r="F31" s="11" t="n">
         <f aca="false">F7+F8+F10+F12+F13+F14+F15+F16+F17+F18+F19+F21+F22+F24+F25+F26+F27</f>
         <v>14900000</v>
       </c>
-      <c r="G31" s="17" t="n">
+      <c r="G31" s="11" t="n">
         <f aca="false">G7+G8+G10+G12+G13+G14+G15+G16+G17+G18+G19+G21+G22+G24+G25+G26+G27</f>
-        <v>10005000</v>
+        <v>10605000</v>
       </c>
     </row>
   </sheetData>
@@ -4541,21 +4516,21 @@
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="12" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>168</v>
@@ -4567,153 +4542,153 @@
         <v>170</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="6" t="n">
         <f aca="false">'PBC Personnel'!L57</f>
         <v>5257000</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="6" t="n">
         <f aca="false">'PBC Personnel'!M57</f>
         <v>7273000</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="6" t="n">
         <f aca="false">'PBC Personnel'!N57</f>
         <v>7831250</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="6" t="n">
         <f aca="false">'PBC Operations'!B11</f>
         <v>1900000</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="6" t="n">
         <f aca="false">'PBC Operations'!C11</f>
         <v>4300000</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="6" t="n">
         <f aca="false">'PBC Operations'!D11</f>
         <v>3100000</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="9" t="n">
         <f aca="false">B6+B7</f>
         <v>7157000</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="9" t="n">
         <f aca="false">C6+C7</f>
         <v>11573000</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="9" t="n">
         <f aca="false">D6+D7</f>
         <v>10931250</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="6" t="n">
         <f aca="false">'PBC Revenue'!E30</f>
-        <v>750000</v>
-      </c>
-      <c r="C11" s="13" t="n">
+        <v>900000</v>
+      </c>
+      <c r="C11" s="6" t="n">
         <f aca="false">'PBC Revenue'!F30</f>
         <v>2200000</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="6" t="n">
         <f aca="false">'PBC Revenue'!G30</f>
-        <v>1475000</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
+        <v>1550000</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="6" t="n">
         <f aca="false">'PBC Revenue'!E31</f>
-        <v>5110000</v>
-      </c>
-      <c r="C12" s="13" t="n">
+        <v>6310000</v>
+      </c>
+      <c r="C12" s="6" t="n">
         <f aca="false">'PBC Revenue'!F31</f>
         <v>14900000</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="6" t="n">
         <f aca="false">'PBC Revenue'!G31</f>
-        <v>10005000</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+        <v>10605000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="9" t="n">
         <f aca="false">B11+B12+B13</f>
-        <v>5860000</v>
-      </c>
-      <c r="C14" s="15" t="n">
+        <v>7210000</v>
+      </c>
+      <c r="C14" s="9" t="n">
         <f aca="false">C11+C12+C13</f>
         <v>17100000</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="9" t="n">
         <f aca="false">D11+D12+D13</f>
-        <v>11480000</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+        <v>12155000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="9" t="n">
         <f aca="false">B14-B8</f>
-        <v>-1297000</v>
-      </c>
-      <c r="C16" s="15" t="n">
+        <v>53000</v>
+      </c>
+      <c r="C16" s="9" t="n">
         <f aca="false">C14-C8</f>
         <v>5527000</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="9" t="n">
         <f aca="false">D14-D8</f>
-        <v>548750</v>
+        <v>1223750</v>
       </c>
     </row>
   </sheetData>

</xml_diff>